<commit_message>
Atualização do relatório de vendas com formatação profissional
</commit_message>
<xml_diff>
--- a/Relatorio_Vendas_Limpo.xlsx
+++ b/Relatorio_Vendas_Limpo.xlsx
@@ -16,11 +16,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="167" formatCode="R$ #,##0.00"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,13 +30,26 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004F81BD"/>
+        <bgColor rgb="004F81BD"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,9 +64,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,46 +439,55 @@
   </sheetPr>
   <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Produto</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Quantidade</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Preço</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Vendedor</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>45297</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -474,7 +503,7 @@
       <c r="D2" t="n">
         <v>5</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="3" t="n">
         <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
@@ -482,12 +511,12 @@
           <t>Ana</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="3" t="n">
         <v>5000</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>45319</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -503,7 +532,7 @@
       <c r="D3" t="n">
         <v>5</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="3" t="n">
         <v>100</v>
       </c>
       <c r="F3" t="inlineStr">
@@ -511,12 +540,12 @@
           <t>Carlos</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="3" t="n">
         <v>500</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>45348</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -532,7 +561,7 @@
       <c r="D4" t="n">
         <v>4</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="3" t="n">
         <v>1278</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -540,12 +569,12 @@
           <t>Carlos</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="3" t="n">
         <v>5112</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>45340</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -561,7 +590,7 @@
       <c r="D5" t="n">
         <v>4</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="3" t="n">
         <v>500</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -569,12 +598,12 @@
           <t>Ana</t>
         </is>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="3" t="n">
         <v>2000</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>45339</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -590,7 +619,7 @@
       <c r="D6" t="n">
         <v>2</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6" s="3" t="n">
         <v>1122</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -598,22 +627,22 @@
           <t>Ana</t>
         </is>
       </c>
-      <c r="G6" t="n">
+      <c r="G6" s="3" t="n">
         <v>2244</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Faturamento Total</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="3" t="n">
         <v>14856</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Produto mais Vendido</t>
         </is>
@@ -628,7 +657,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Vendedor Top</t>
         </is>
@@ -638,7 +667,7 @@
           <t>Ana</t>
         </is>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" s="3" t="n">
         <v>9244</v>
       </c>
     </row>

</xml_diff>